<commit_message>
Update Table2 baseline and ablation configurations
</commit_message>
<xml_diff>
--- a/information/Table2. Configurations of baseline and ablation models.xlsx
+++ b/information/Table2. Configurations of baseline and ablation models.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\研二\免疫治疗模型\github\information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92B3674-EFEF-45F6-9357-DA980187FD4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86E50E9-7626-4515-9BC9-9D16857565C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="44">
   <si>
     <t>Comparison model</t>
   </si>
@@ -114,9 +114,6 @@
     <t>Same 5-fold CV as CoMET; batch size 45, 50 epochs, patience 13, threshold 0.5.</t>
   </si>
   <si>
-    <t>Same 5-fold CV as CoMET; batch size 45, 50 epochs, patience 13, threshold 0.6.</t>
-  </si>
-  <si>
     <t>Independent cohort-specific DNN; 64 → 32 → 16 → 1 with batch normalization, ReLU, and 0.4 dropout.</t>
   </si>
   <si>
@@ -135,9 +132,6 @@
     <t>Uses TCGA-pretrained RNA and shared-encoder parameters; pretrained experts are frozen and MMoE gates are fine-tuned.</t>
   </si>
   <si>
-    <t>Joint 5-fold cohort × response stratified CV; up to 50 epochs, patience = 15, threshold = 0.5.</t>
-  </si>
-  <si>
     <t>Uses the same shared and cohort-specific inputs as CoMET.</t>
   </si>
   <si>
@@ -154,10 +148,23 @@
     <t>No TCGA-pretrained RNA or MMoE parameters are used; the MMoE and task heads are trained from scratch.</t>
   </si>
   <si>
-    <t>Joint 5-fold cohort × response stratified CV; AdamW (lr = 1 × 10⁻⁴), up to 50 epochs, patience = 10, threshold = 0.5.</t>
-  </si>
-  <si>
-    <t>Same as CoMET</t>
+    <t>Using the same 5-fold CV splits as CoMET;  threshold = 0.5.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Joint 5-fold cohort × response stratified CV; up to 50 epochs, patience = 13, threshold = 0.5.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Uses the TCGA-pretrained RNA encoder only; no MMoE parameters are transferred.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Independent 5-fold response-stratified CV within each cohort; up to 50 epochs, patience = 13, threshold = 0.5.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Same 5-fold CV as CoMET; batch size 45, 50 epochs, patience 13, threshold 0.5.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -530,7 +537,7 @@
         <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -547,7 +554,7 @@
         <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -564,7 +571,7 @@
         <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -572,16 +579,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="D5" t="s">
-        <v>34</v>
-      </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -592,13 +599,13 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -609,10 +616,13 @@
         <v>21</v>
       </c>
       <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
         <v>30</v>
       </c>
-      <c r="D7" t="s">
-        <v>31</v>
+      <c r="E7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -620,16 +630,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
         <v>36</v>
       </c>
-      <c r="C8" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" t="s">
-        <v>38</v>
-      </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -637,16 +647,16 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" t="s">
         <v>40</v>
-      </c>
-      <c r="E9" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -680,7 +690,7 @@
         <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>